<commit_message>
Improve CLI, fix test
</commit_message>
<xml_diff>
--- a/tests/test_dataset/RepTest_correct.xlsx
+++ b/tests/test_dataset/RepTest_correct.xlsx
@@ -1,28 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\llenezet\repositories\Files2DB\tests\test_dataset\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C273316-BA0C-45E5-A5B6-66F6498228E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Files" sheetId="1" r:id="rId1"/>
-    <sheet name="FieldRules" sheetId="2" r:id="rId2"/>
-    <sheet name="ValuesMap" sheetId="3" r:id="rId3"/>
+    <sheet name="Files" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="FieldsRules" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="ValuesMap" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="100">
   <si>
     <t>EmplacementOrigine</t>
   </si>
@@ -285,6 +281,12 @@
     <t>A,B,C,D,E</t>
   </si>
   <si>
+    <t>OriginalValues</t>
+  </si>
+  <si>
+    <t>NewValue</t>
+  </si>
+  <si>
     <t>mâle,male,m,</t>
   </si>
   <si>
@@ -316,27 +318,21 @@
   </si>
   <si>
     <t>LabxGol</t>
-  </si>
-  <si>
-    <t>NewValue</t>
-  </si>
-  <si>
-    <t>OriginalValues</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="2">
     <font>
-      <sz val="11"/>
+      <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
     </font>
@@ -349,172 +345,150 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="8">
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
     <border>
       <left style="medium">
-        <color indexed="64"/>
+        <color auto="1"/>
       </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="medium">
         <color auto="1"/>
       </right>
       <top style="medium">
-        <color indexed="64"/>
+        <color auto="1"/>
       </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
     <border>
       <left style="medium">
-        <color indexed="64"/>
+        <color auto="1"/>
       </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="medium">
         <color auto="1"/>
       </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="none"/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
   <cellXfs count="20">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="3" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="0" borderId="1" numFmtId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="0" borderId="2" numFmtId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="0" borderId="3" numFmtId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="3" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="1" fillId="0" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="0" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="0" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="0" borderId="6" numFmtId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="0" borderId="5" numFmtId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="0" borderId="7" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="0" borderId="3" numFmtId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -534,8 +508,291 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Angsana New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Cordia New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -749,39 +1006,38 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <outlinePr summaryBelow="0"/>
+    <outlinePr applyStyles="0" summaryBelow="0" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:T3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="45.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="7.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="6.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col bestFit="1" customWidth="1" min="1" max="1" width="19.85546875"/>
+    <col bestFit="1" customWidth="1" min="2" max="2" width="14.5703125"/>
+    <col bestFit="1" customWidth="1" min="3" max="3" width="9.5703125"/>
+    <col bestFit="1" customWidth="1" min="4" max="4" width="45.42578125"/>
+    <col bestFit="1" customWidth="1" min="5" max="5" width="11.42578125"/>
+    <col bestFit="1" customWidth="1" min="6" max="6" width="8.85546875"/>
+    <col bestFit="1" customWidth="1" min="7" max="7" width="8"/>
+    <col bestFit="1" customWidth="1" min="8" max="8" width="7.42578125"/>
+    <col bestFit="1" customWidth="1" min="9" max="9" style="1" width="8"/>
+    <col bestFit="1" customWidth="1" min="10" max="11" style="1" width="7.140625"/>
+    <col bestFit="1" customWidth="1" min="12" max="12" width="8.7109375"/>
+    <col bestFit="1" customWidth="1" min="13" max="13" width="16.140625"/>
+    <col bestFit="1" customWidth="1" min="14" max="14" style="1" width="8.42578125"/>
+    <col bestFit="1" customWidth="1" min="15" max="15" style="1" width="6.7109375"/>
+    <col bestFit="1" customWidth="1" min="16" max="16" style="1" width="12.42578125"/>
+    <col bestFit="1" customWidth="1" min="17" max="17" width="20.28515625"/>
+    <col bestFit="1" customWidth="1" min="18" max="18" width="5.85546875"/>
+    <col bestFit="1" customWidth="1" min="19" max="19" width="12.7109375"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="18.75" customHeight="1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -843,7 +1099,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:20" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" ht="18.75" customHeight="1">
       <c r="A2" t="s">
         <v>20</v>
       </c>
@@ -890,7 +1146,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3">
       <c r="A3" t="s">
         <v>29</v>
       </c>
@@ -923,32 +1179,34 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <outlinePr summaryBelow="0"/>
+    <outlinePr applyStyles="0" summaryBelow="0" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="27.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="5" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.5703125" customWidth="1"/>
-    <col min="7" max="7" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="18.42578125" style="7" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="68.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="16.140625" bestFit="1" customWidth="1"/>
+    <col bestFit="1" customWidth="1" min="1" max="1" width="27.140625"/>
+    <col bestFit="1" customWidth="1" min="2" max="5" width="13.5703125"/>
+    <col customWidth="1" min="6" max="6" width="13.5703125"/>
+    <col bestFit="1" customWidth="1" min="7" max="7" width="13.5703125"/>
+    <col bestFit="1" customWidth="1" min="8" max="8" width="22.28515625"/>
+    <col bestFit="1" customWidth="1" min="9" max="10" width="13.5703125"/>
+    <col bestFit="1" customWidth="1" min="11" max="12" style="7" width="18.42578125"/>
+    <col bestFit="1" customWidth="1" min="13" max="13" width="68.85546875"/>
+    <col bestFit="1" customWidth="1" min="14" max="14" width="9.42578125"/>
+    <col bestFit="1" customWidth="1" min="15" max="15" width="16.140625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="18.75" customHeight="1">
       <c r="A1" s="8" t="s">
         <v>34</v>
       </c>
@@ -995,7 +1253,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" ht="18.75" customHeight="1">
       <c r="A2" s="13" t="s">
         <v>49</v>
       </c>
@@ -1021,7 +1279,7 @@
       <c r="M2" s="15"/>
       <c r="N2" s="16"/>
     </row>
-    <row r="3" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" ht="18.75" customHeight="1">
       <c r="A3" s="13" t="s">
         <v>56</v>
       </c>
@@ -1041,7 +1299,7 @@
       <c r="M3" s="15"/>
       <c r="N3" s="16"/>
     </row>
-    <row r="4" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" ht="18.75" customHeight="1">
       <c r="A4" s="13" t="s">
         <v>60</v>
       </c>
@@ -1064,7 +1322,7 @@
       <c r="M4" s="15"/>
       <c r="N4" s="16"/>
     </row>
-    <row r="5" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" ht="18.75" customHeight="1">
       <c r="A5" s="13" t="s">
         <v>63</v>
       </c>
@@ -1094,7 +1352,7 @@
       <c r="M5" s="15"/>
       <c r="N5" s="16"/>
     </row>
-    <row r="6" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" ht="18.75" customHeight="1">
       <c r="A6" s="13" t="s">
         <v>68</v>
       </c>
@@ -1117,7 +1375,7 @@
       <c r="L6" s="17"/>
       <c r="N6" s="14"/>
     </row>
-    <row r="7" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" ht="18.75" customHeight="1">
       <c r="A7" s="13" t="s">
         <v>73</v>
       </c>
@@ -1141,7 +1399,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" ht="18.75" customHeight="1">
       <c r="A8" s="13" t="s">
         <v>78</v>
       </c>
@@ -1169,7 +1427,7 @@
       <c r="M8" s="15"/>
       <c r="N8" s="16"/>
     </row>
-    <row r="9" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" ht="18.75" customHeight="1">
       <c r="A9" s="13" t="s">
         <v>79</v>
       </c>
@@ -1197,7 +1455,7 @@
       <c r="M9" s="15"/>
       <c r="N9" s="16"/>
     </row>
-    <row r="10" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" ht="18.75" customHeight="1">
       <c r="A10" s="13" t="s">
         <v>81</v>
       </c>
@@ -1218,7 +1476,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11">
       <c r="A11" s="13" t="s">
         <v>85</v>
       </c>
@@ -1238,101 +1496,105 @@
       <c r="N11" s="16"/>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <outlinePr summaryBelow="0"/>
+    <outlinePr applyStyles="0" summaryBelow="0" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" style="18" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" style="18" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.5703125" style="18" bestFit="1" customWidth="1"/>
+    <col bestFit="1" customWidth="1" min="1" max="1" style="18" width="13.5703125"/>
+    <col bestFit="1" customWidth="1" min="2" max="2" style="18" width="16.42578125"/>
+    <col bestFit="1" customWidth="1" min="3" max="3" style="18" width="13.5703125"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="18.75" customHeight="1">
       <c r="A1" s="18" t="s">
         <v>34</v>
       </c>
       <c r="B1" s="18" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="C1" s="18" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" s="18" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="2" s="18" customFormat="1" ht="18.75" customHeight="1">
       <c r="A2" s="19" t="s">
         <v>56</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" s="18" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="3" s="18" customFormat="1" ht="18.75" customHeight="1">
       <c r="A3" s="19" t="s">
         <v>56</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C3" s="19" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" s="18" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="4" s="18" customFormat="1" ht="18.75" customHeight="1">
       <c r="A4" s="19" t="s">
         <v>56</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C4" s="19"/>
     </row>
-    <row r="5" spans="1:3" s="18" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" s="18" customFormat="1" ht="18.75" customHeight="1">
       <c r="A5" s="19" t="s">
         <v>60</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" s="18" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="6" s="18" customFormat="1" ht="18.75" customHeight="1">
       <c r="A6" s="19" t="s">
         <v>60</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" s="18" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="7" s="18" customFormat="1" ht="18.75" customHeight="1">
       <c r="A7" s="19" t="s">
         <v>60</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>